<commit_message>
feat: registrar 11-E-9770-02 TRTC y 11-A-9581-01 TRTC en catálogo, SKUs autorizados e imágenes
</commit_message>
<xml_diff>
--- a/BD_Articulos.xlsx
+++ b/BD_Articulos.xlsx
@@ -1,13 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Datos_Sistema" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -50,7 +49,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -413,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F528"/>
+  <dimension ref="A1:F534"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -646,9 +645,6 @@
           <t>11-A-6013-01</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -666,9 +662,6 @@
           <t>11-A-6013-03</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -792,7 +785,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -820,7 +812,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -838,9 +829,6 @@
           <t>11-A-6102-01</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -858,9 +846,6 @@
           <t>11-A-9012-01</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -878,9 +863,6 @@
           <t>11-A-9023-01</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -898,9 +880,6 @@
           <t>11-A-9024-01</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -918,9 +897,6 @@
           <t>11-A-9025-01</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -938,9 +914,6 @@
           <t>11-A-9026-01</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -958,9 +931,6 @@
           <t>11-A-9027-01</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -978,9 +948,6 @@
           <t>11-A-9028-01</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -998,9 +965,6 @@
           <t>11-A-9029-01</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1018,9 +982,6 @@
           <t>11-A-9029-02</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1038,9 +999,6 @@
           <t>11-A-9030-01</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1058,9 +1016,6 @@
           <t>11-A-9030-02</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1078,9 +1033,6 @@
           <t>11-A-9040-01</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1098,9 +1050,6 @@
           <t>11-A-9577-01</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1118,9 +1067,16 @@
           <t>11-A-9581-01</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RUN-BACK LUG BRACKET</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Decapado CAL 16 (16 GA)</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1138,9 +1094,6 @@
           <t>11-A-9582-01</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1158,9 +1111,6 @@
           <t>11-A-9794-01</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1178,9 +1128,6 @@
           <t>11-A-9795-01</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1198,9 +1145,6 @@
           <t>11-A-9804-01</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1218,9 +1162,6 @@
           <t>11-A-9807-01</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1238,9 +1179,6 @@
           <t>11-A-9813-01</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1258,9 +1196,6 @@
           <t>11-A-9813-02</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1278,9 +1213,6 @@
           <t>11-A-9815-01</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1298,9 +1230,6 @@
           <t>11-A-9816-01</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1318,9 +1247,6 @@
           <t>11-A-9830-01</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1338,9 +1264,6 @@
           <t>11-A-9836-01</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1358,9 +1281,6 @@
           <t>11-A-9837-01</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1378,9 +1298,6 @@
           <t>11-A-9843-01</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1398,9 +1315,6 @@
           <t>11-A-9845-01</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1418,9 +1332,6 @@
           <t>11-A-9846-01</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1438,9 +1349,6 @@
           <t>11-A-9847-01</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1458,9 +1366,6 @@
           <t>11-A-9853-01</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1478,9 +1383,6 @@
           <t>11-A-9875-01</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1498,9 +1400,6 @@
           <t>11-A-9875-03</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1518,9 +1417,6 @@
           <t>11-A-9875-07</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1538,9 +1434,6 @@
           <t>11-A-9895-01</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1558,9 +1451,6 @@
           <t>11-A-9897-01</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1578,9 +1468,6 @@
           <t>11-A-9908-01</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1598,9 +1485,6 @@
           <t>11-A-9909-01</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1618,9 +1502,6 @@
           <t>11-A-9916-01</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1638,9 +1519,6 @@
           <t>11-A-9917-01</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1658,13 +1536,11 @@
           <t>11-A-9921-01</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1682,13 +1558,11 @@
           <t>11-A-9923-01</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1706,9 +1580,6 @@
           <t>11-A-9925-01</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1726,9 +1597,6 @@
           <t>11-A-9926-01</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1746,9 +1614,6 @@
           <t>11-A-9927-01</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1766,9 +1631,6 @@
           <t>11-A-9951-01</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1786,9 +1648,6 @@
           <t>11-A-9958-01</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1806,9 +1665,6 @@
           <t>11-A-9959-01</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1826,9 +1682,6 @@
           <t>11-A-9960-01</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1846,9 +1699,6 @@
           <t>11-A-9961-01</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1866,9 +1716,6 @@
           <t>11-A-9983-01</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1918,9 +1765,6 @@
           <t>11-B-9034-01</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1938,9 +1782,6 @@
           <t>11-B-9074-01</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1958,9 +1799,6 @@
           <t>11-B-9079-01</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1978,9 +1816,6 @@
           <t>11-B-9083-01</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -1998,9 +1833,6 @@
           <t>11-B-9085-01</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr"/>
-      <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2018,9 +1850,6 @@
           <t>11-B-9086-01</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2038,9 +1867,6 @@
           <t>11-B-9088-01</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr"/>
-      <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2058,9 +1884,6 @@
           <t>11-B-9123-01</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2078,13 +1901,11 @@
           <t>11-B-9126-01</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2102,13 +1923,11 @@
           <t>11-B-9127-01</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2126,9 +1945,6 @@
           <t>11-B-9147-01</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr"/>
-      <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2146,9 +1962,6 @@
           <t>11-B-9193-01</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr"/>
-      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2166,9 +1979,6 @@
           <t>11-B-9194-03</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr"/>
-      <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2186,9 +1996,6 @@
           <t>11-B-9194-04</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2206,9 +2013,6 @@
           <t>11-B-9195-01</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr"/>
-      <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2226,9 +2030,6 @@
           <t>11-B-9208-01</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr"/>
-      <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2246,9 +2047,6 @@
           <t>11-B-9208-02</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr"/>
-      <c r="C84" t="inlineStr"/>
-      <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2266,9 +2064,6 @@
           <t>11-B-9211-01</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr"/>
-      <c r="C85" t="inlineStr"/>
-      <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2286,9 +2081,6 @@
           <t>11-B-9310-01</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
-      <c r="C86" t="inlineStr"/>
-      <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2306,9 +2098,6 @@
           <t>11-B-9311-02</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
-      <c r="C87" t="inlineStr"/>
-      <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2326,9 +2115,6 @@
           <t>11-B-9362-01</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr"/>
-      <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2346,9 +2132,6 @@
           <t>11-B-9374-01</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
-      <c r="C89" t="inlineStr"/>
-      <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2366,9 +2149,6 @@
           <t>11-B-9411-01</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
-      <c r="C90" t="inlineStr"/>
-      <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2386,9 +2166,6 @@
           <t>11-B-9520-01</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr"/>
-      <c r="C91" t="inlineStr"/>
-      <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2406,9 +2183,6 @@
           <t>11-B-9521-01</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
-      <c r="C92" t="inlineStr"/>
-      <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2426,9 +2200,6 @@
           <t>11-B-9528-01</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr"/>
-      <c r="C93" t="inlineStr"/>
-      <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2446,9 +2217,6 @@
           <t>11-B-9618-01</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr"/>
-      <c r="C94" t="inlineStr"/>
-      <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2466,9 +2234,6 @@
           <t>11-B-9620-01</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr"/>
-      <c r="C95" t="inlineStr"/>
-      <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2486,9 +2251,6 @@
           <t>11-B-9697-01</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr"/>
-      <c r="C96" t="inlineStr"/>
-      <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2506,9 +2268,6 @@
           <t>11-B-9743-01</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr"/>
-      <c r="D97" t="inlineStr"/>
       <c r="E97" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2526,9 +2285,6 @@
           <t>11-B-9743-02</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr"/>
-      <c r="C98" t="inlineStr"/>
-      <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2546,9 +2302,6 @@
           <t>11-B-9753-01</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr"/>
-      <c r="C99" t="inlineStr"/>
-      <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2566,9 +2319,6 @@
           <t>11-B-9754-01</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr"/>
-      <c r="C100" t="inlineStr"/>
-      <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2586,9 +2336,6 @@
           <t>11-B-9754-02</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr"/>
-      <c r="C101" t="inlineStr"/>
-      <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2606,9 +2353,6 @@
           <t>11-B-9755-01</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr"/>
-      <c r="C102" t="inlineStr"/>
-      <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2658,9 +2402,6 @@
           <t>11-C-9115-01</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr"/>
-      <c r="C104" t="inlineStr"/>
-      <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2678,9 +2419,6 @@
           <t>11-C-9115-02</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr"/>
-      <c r="C105" t="inlineStr"/>
-      <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2698,9 +2436,6 @@
           <t>11-C-9229-01</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr"/>
-      <c r="C106" t="inlineStr"/>
-      <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2718,9 +2453,6 @@
           <t>11-C-9230-01</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr"/>
-      <c r="C107" t="inlineStr"/>
-      <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2738,9 +2470,6 @@
           <t>11-C-9231-01</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr"/>
-      <c r="C108" t="inlineStr"/>
-      <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2758,9 +2487,6 @@
           <t>11-C-9232-01</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr"/>
-      <c r="C109" t="inlineStr"/>
-      <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2778,9 +2504,6 @@
           <t>11-C-9233-01</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr"/>
-      <c r="C110" t="inlineStr"/>
-      <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2798,9 +2521,6 @@
           <t>11-C-9233-02</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr"/>
-      <c r="C111" t="inlineStr"/>
-      <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2818,13 +2538,11 @@
           <t>11-C-9241-01</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr"/>
       <c r="C112" t="inlineStr">
         <is>
           <t>14GACR</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2842,13 +2560,11 @@
           <t>11-C-9241-02</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr"/>
       <c r="C113" t="inlineStr">
         <is>
           <t>14GACR</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2866,13 +2582,11 @@
           <t>11-C-9242-01</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr"/>
       <c r="C114" t="inlineStr">
         <is>
           <t>14GACR</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2890,13 +2604,11 @@
           <t>11-C-9242-02</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr"/>
       <c r="C115" t="inlineStr">
         <is>
           <t>14GACR</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2914,9 +2626,6 @@
           <t>11-C-9243-01</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr"/>
-      <c r="C116" t="inlineStr"/>
-      <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2934,13 +2643,11 @@
           <t>11-C-9244-01</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr"/>
       <c r="C117" t="inlineStr">
         <is>
           <t>14GACR</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2958,9 +2665,6 @@
           <t>11-C-9245-01</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr"/>
-      <c r="C118" t="inlineStr"/>
-      <c r="D118" t="inlineStr"/>
       <c r="E118" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2978,9 +2682,6 @@
           <t>11-C-9246-01</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr"/>
-      <c r="C119" t="inlineStr"/>
-      <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -2998,13 +2699,11 @@
           <t>11-C-9247-01</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr"/>
       <c r="C120" t="inlineStr">
         <is>
           <t>14GACR</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3022,13 +2721,11 @@
           <t>11-C-9248-01</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr"/>
       <c r="C121" t="inlineStr">
         <is>
           <t>14GACR</t>
         </is>
       </c>
-      <c r="D121" t="inlineStr"/>
       <c r="E121" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3046,9 +2743,6 @@
           <t>11-C-9249-01</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr"/>
-      <c r="C122" t="inlineStr"/>
-      <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3066,9 +2760,6 @@
           <t>11-C-9250-01</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr"/>
-      <c r="C123" t="inlineStr"/>
-      <c r="D123" t="inlineStr"/>
       <c r="E123" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3086,9 +2777,6 @@
           <t>11-C-9277-02</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr"/>
-      <c r="C124" t="inlineStr"/>
-      <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3106,9 +2794,6 @@
           <t>11-C-9280-01</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr"/>
-      <c r="C125" t="inlineStr"/>
-      <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3126,9 +2811,6 @@
           <t>11-C-9281-01</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr"/>
-      <c r="C126" t="inlineStr"/>
-      <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3146,9 +2828,6 @@
           <t>11-C-9282-01</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr"/>
-      <c r="C127" t="inlineStr"/>
-      <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3166,9 +2845,6 @@
           <t>11-C-9283-01</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr"/>
-      <c r="C128" t="inlineStr"/>
-      <c r="D128" t="inlineStr"/>
       <c r="E128" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3186,9 +2862,6 @@
           <t>11-C-9284-01</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr"/>
-      <c r="C129" t="inlineStr"/>
-      <c r="D129" t="inlineStr"/>
       <c r="E129" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3206,9 +2879,6 @@
           <t>11-C-9285-01</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr"/>
-      <c r="C130" t="inlineStr"/>
-      <c r="D130" t="inlineStr"/>
       <c r="E130" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3226,13 +2896,11 @@
           <t>11-C-9300-01</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr"/>
       <c r="C131" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D131" t="inlineStr"/>
       <c r="E131" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3250,13 +2918,11 @@
           <t>11-C-9307-01</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr"/>
       <c r="C132" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D132" t="inlineStr"/>
       <c r="E132" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3274,13 +2940,11 @@
           <t>11-C-9333-01</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr"/>
       <c r="C133" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D133" t="inlineStr"/>
       <c r="E133" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3298,13 +2962,11 @@
           <t>11-C-9352-01</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr"/>
       <c r="C134" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D134" t="inlineStr"/>
       <c r="E134" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3322,9 +2984,6 @@
           <t>11-C-9576-02</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr"/>
-      <c r="C135" t="inlineStr"/>
-      <c r="D135" t="inlineStr"/>
       <c r="E135" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3342,9 +3001,6 @@
           <t>11-C-9582-01</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr"/>
-      <c r="C136" t="inlineStr"/>
-      <c r="D136" t="inlineStr"/>
       <c r="E136" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3362,13 +3018,11 @@
           <t>11-C-9611-01</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr"/>
       <c r="C137" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D137" t="inlineStr"/>
       <c r="E137" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3386,13 +3040,11 @@
           <t>11-C-9612-01</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr"/>
       <c r="C138" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D138" t="inlineStr"/>
       <c r="E138" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3410,13 +3062,11 @@
           <t>11-C-9617-01</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr"/>
       <c r="C139" t="inlineStr">
         <is>
           <t>14GACR</t>
         </is>
       </c>
-      <c r="D139" t="inlineStr"/>
       <c r="E139" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3434,13 +3084,11 @@
           <t>11-C-9618-01</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr"/>
       <c r="C140" t="inlineStr">
         <is>
           <t>14GACR</t>
         </is>
       </c>
-      <c r="D140" t="inlineStr"/>
       <c r="E140" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3458,9 +3106,6 @@
           <t>11-C-9620-01</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr"/>
-      <c r="C141" t="inlineStr"/>
-      <c r="D141" t="inlineStr"/>
       <c r="E141" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3478,9 +3123,6 @@
           <t>11-C-9621-01</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr"/>
-      <c r="C142" t="inlineStr"/>
-      <c r="D142" t="inlineStr"/>
       <c r="E142" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3498,13 +3140,11 @@
           <t>11-C-9634-01</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr"/>
       <c r="C143" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D143" t="inlineStr"/>
       <c r="E143" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3522,13 +3162,11 @@
           <t>11-C-9638-01</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr"/>
       <c r="C144" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D144" t="inlineStr"/>
       <c r="E144" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3546,13 +3184,11 @@
           <t>11-C-9639-01</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr"/>
       <c r="C145" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D145" t="inlineStr"/>
       <c r="E145" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3570,13 +3206,11 @@
           <t>11-C-9639-02</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr"/>
       <c r="C146" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D146" t="inlineStr"/>
       <c r="E146" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3594,9 +3228,6 @@
           <t>11-C-9665-01</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr"/>
-      <c r="C147" t="inlineStr"/>
-      <c r="D147" t="inlineStr"/>
       <c r="E147" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3614,9 +3245,6 @@
           <t>11-C-9666-01</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr"/>
-      <c r="C148" t="inlineStr"/>
-      <c r="D148" t="inlineStr"/>
       <c r="E148" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3634,13 +3262,11 @@
           <t>11-C-9669-01</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr"/>
       <c r="C149" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D149" t="inlineStr"/>
       <c r="E149" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3658,13 +3284,11 @@
           <t>11-C-9681-01</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr"/>
       <c r="C150" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D150" t="inlineStr"/>
       <c r="E150" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3682,13 +3306,11 @@
           <t>11-C-9681-02</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr"/>
       <c r="C151" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr"/>
       <c r="E151" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3706,9 +3328,6 @@
           <t>11-C-9708-01</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr"/>
-      <c r="C152" t="inlineStr"/>
-      <c r="D152" t="inlineStr"/>
       <c r="E152" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3726,9 +3345,6 @@
           <t>11-C-9709-01</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr"/>
-      <c r="C153" t="inlineStr"/>
-      <c r="D153" t="inlineStr"/>
       <c r="E153" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3746,9 +3362,6 @@
           <t>11-C-9746-01</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr"/>
-      <c r="C154" t="inlineStr"/>
-      <c r="D154" t="inlineStr"/>
       <c r="E154" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3766,9 +3379,6 @@
           <t>11-C-9747-01</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr"/>
-      <c r="C155" t="inlineStr"/>
-      <c r="D155" t="inlineStr"/>
       <c r="E155" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3786,9 +3396,6 @@
           <t>11-C-9778-01</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr"/>
-      <c r="C156" t="inlineStr"/>
-      <c r="D156" t="inlineStr"/>
       <c r="E156" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3806,9 +3413,6 @@
           <t>11-C-9779-01</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr"/>
-      <c r="C157" t="inlineStr"/>
-      <c r="D157" t="inlineStr"/>
       <c r="E157" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3826,9 +3430,6 @@
           <t>11-C-9831-01</t>
         </is>
       </c>
-      <c r="B158" t="inlineStr"/>
-      <c r="C158" t="inlineStr"/>
-      <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3846,9 +3447,6 @@
           <t>11-C-9832-01</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr"/>
-      <c r="C159" t="inlineStr"/>
-      <c r="D159" t="inlineStr"/>
       <c r="E159" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3866,9 +3464,6 @@
           <t>11-C-9924-01</t>
         </is>
       </c>
-      <c r="B160" t="inlineStr"/>
-      <c r="C160" t="inlineStr"/>
-      <c r="D160" t="inlineStr"/>
       <c r="E160" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3886,13 +3481,11 @@
           <t>11-C-9926-01</t>
         </is>
       </c>
-      <c r="B161" t="inlineStr"/>
       <c r="C161" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D161" t="inlineStr"/>
       <c r="E161" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3910,13 +3503,11 @@
           <t>11-C-9943-02</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr"/>
       <c r="C162" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3934,13 +3525,11 @@
           <t>11-C-9944-01</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr"/>
       <c r="C163" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D163" t="inlineStr"/>
       <c r="E163" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3958,9 +3547,6 @@
           <t>11-C-9962-01</t>
         </is>
       </c>
-      <c r="B164" t="inlineStr"/>
-      <c r="C164" t="inlineStr"/>
-      <c r="D164" t="inlineStr"/>
       <c r="E164" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -3978,9 +3564,6 @@
           <t>11-C-9977-01</t>
         </is>
       </c>
-      <c r="B165" t="inlineStr"/>
-      <c r="C165" t="inlineStr"/>
-      <c r="D165" t="inlineStr"/>
       <c r="E165" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4003,8 +3586,6 @@
           <t>11-D-3385-01-(16gacr ANSI-61) - K48 - V0-R0</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr"/>
-      <c r="D166" t="inlineStr"/>
       <c r="E166" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4128,7 +3709,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D170" t="inlineStr"/>
       <c r="E170" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -4210,9 +3790,6 @@
           <t>11-D-6245-02</t>
         </is>
       </c>
-      <c r="B173" t="inlineStr"/>
-      <c r="C173" t="inlineStr"/>
-      <c r="D173" t="inlineStr"/>
       <c r="E173" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4230,9 +3807,6 @@
           <t>11-D-6246-03</t>
         </is>
       </c>
-      <c r="B174" t="inlineStr"/>
-      <c r="C174" t="inlineStr"/>
-      <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4250,9 +3824,6 @@
           <t>11-D-6246-04</t>
         </is>
       </c>
-      <c r="B175" t="inlineStr"/>
-      <c r="C175" t="inlineStr"/>
-      <c r="D175" t="inlineStr"/>
       <c r="E175" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4270,9 +3841,6 @@
           <t>11-D-6252-03</t>
         </is>
       </c>
-      <c r="B176" t="inlineStr"/>
-      <c r="C176" t="inlineStr"/>
-      <c r="D176" t="inlineStr"/>
       <c r="E176" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4290,9 +3858,6 @@
           <t>11-D-6252-05</t>
         </is>
       </c>
-      <c r="B177" t="inlineStr"/>
-      <c r="C177" t="inlineStr"/>
-      <c r="D177" t="inlineStr"/>
       <c r="E177" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4310,9 +3875,6 @@
           <t>11-D-9004-01</t>
         </is>
       </c>
-      <c r="B178" t="inlineStr"/>
-      <c r="C178" t="inlineStr"/>
-      <c r="D178" t="inlineStr"/>
       <c r="E178" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4330,9 +3892,6 @@
           <t>11-D-9146-01</t>
         </is>
       </c>
-      <c r="B179" t="inlineStr"/>
-      <c r="C179" t="inlineStr"/>
-      <c r="D179" t="inlineStr"/>
       <c r="E179" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4350,9 +3909,6 @@
           <t>11-D-9156-01</t>
         </is>
       </c>
-      <c r="B180" t="inlineStr"/>
-      <c r="C180" t="inlineStr"/>
-      <c r="D180" t="inlineStr"/>
       <c r="E180" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4370,9 +3926,6 @@
           <t>11-D-9156-04</t>
         </is>
       </c>
-      <c r="B181" t="inlineStr"/>
-      <c r="C181" t="inlineStr"/>
-      <c r="D181" t="inlineStr"/>
       <c r="E181" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4390,9 +3943,6 @@
           <t>11-D-9297-01</t>
         </is>
       </c>
-      <c r="B182" t="inlineStr"/>
-      <c r="C182" t="inlineStr"/>
-      <c r="D182" t="inlineStr"/>
       <c r="E182" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4410,9 +3960,6 @@
           <t>11-D-9298-01</t>
         </is>
       </c>
-      <c r="B183" t="inlineStr"/>
-      <c r="C183" t="inlineStr"/>
-      <c r="D183" t="inlineStr"/>
       <c r="E183" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4430,9 +3977,6 @@
           <t>11-D-9443-01</t>
         </is>
       </c>
-      <c r="B184" t="inlineStr"/>
-      <c r="C184" t="inlineStr"/>
-      <c r="D184" t="inlineStr"/>
       <c r="E184" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4450,9 +3994,6 @@
           <t>11-D-9534-01</t>
         </is>
       </c>
-      <c r="B185" t="inlineStr"/>
-      <c r="C185" t="inlineStr"/>
-      <c r="D185" t="inlineStr"/>
       <c r="E185" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4470,9 +4011,6 @@
           <t>11-D-9535-01</t>
         </is>
       </c>
-      <c r="B186" t="inlineStr"/>
-      <c r="C186" t="inlineStr"/>
-      <c r="D186" t="inlineStr"/>
       <c r="E186" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4490,9 +4028,6 @@
           <t>11-D-9539-01</t>
         </is>
       </c>
-      <c r="B187" t="inlineStr"/>
-      <c r="C187" t="inlineStr"/>
-      <c r="D187" t="inlineStr"/>
       <c r="E187" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4510,9 +4045,6 @@
           <t>11-D-9643-01</t>
         </is>
       </c>
-      <c r="B188" t="inlineStr"/>
-      <c r="C188" t="inlineStr"/>
-      <c r="D188" t="inlineStr"/>
       <c r="E188" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4530,9 +4062,6 @@
           <t>11-D-9643-02</t>
         </is>
       </c>
-      <c r="B189" t="inlineStr"/>
-      <c r="C189" t="inlineStr"/>
-      <c r="D189" t="inlineStr"/>
       <c r="E189" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4550,9 +4079,6 @@
           <t>11-D-9732-01</t>
         </is>
       </c>
-      <c r="B190" t="inlineStr"/>
-      <c r="C190" t="inlineStr"/>
-      <c r="D190" t="inlineStr"/>
       <c r="E190" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4570,9 +4096,6 @@
           <t>11-D-9733-01</t>
         </is>
       </c>
-      <c r="B191" t="inlineStr"/>
-      <c r="C191" t="inlineStr"/>
-      <c r="D191" t="inlineStr"/>
       <c r="E191" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4590,9 +4113,6 @@
           <t>11-D-9736-02</t>
         </is>
       </c>
-      <c r="B192" t="inlineStr"/>
-      <c r="C192" t="inlineStr"/>
-      <c r="D192" t="inlineStr"/>
       <c r="E192" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4610,9 +4130,6 @@
           <t>11-D-9740-01</t>
         </is>
       </c>
-      <c r="B193" t="inlineStr"/>
-      <c r="C193" t="inlineStr"/>
-      <c r="D193" t="inlineStr"/>
       <c r="E193" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4630,9 +4147,6 @@
           <t>11-D-9741-01</t>
         </is>
       </c>
-      <c r="B194" t="inlineStr"/>
-      <c r="C194" t="inlineStr"/>
-      <c r="D194" t="inlineStr"/>
       <c r="E194" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4650,9 +4164,6 @@
           <t>11-D-9742-01</t>
         </is>
       </c>
-      <c r="B195" t="inlineStr"/>
-      <c r="C195" t="inlineStr"/>
-      <c r="D195" t="inlineStr"/>
       <c r="E195" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4670,9 +4181,6 @@
           <t>11-D-9775-01</t>
         </is>
       </c>
-      <c r="B196" t="inlineStr"/>
-      <c r="C196" t="inlineStr"/>
-      <c r="D196" t="inlineStr"/>
       <c r="E196" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4690,9 +4198,6 @@
           <t>11-D-9812-01</t>
         </is>
       </c>
-      <c r="B197" t="inlineStr"/>
-      <c r="C197" t="inlineStr"/>
-      <c r="D197" t="inlineStr"/>
       <c r="E197" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4710,9 +4215,6 @@
           <t>11-D-9814-01</t>
         </is>
       </c>
-      <c r="B198" t="inlineStr"/>
-      <c r="C198" t="inlineStr"/>
-      <c r="D198" t="inlineStr"/>
       <c r="E198" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4730,9 +4232,6 @@
           <t>11-D-9817-01</t>
         </is>
       </c>
-      <c r="B199" t="inlineStr"/>
-      <c r="C199" t="inlineStr"/>
-      <c r="D199" t="inlineStr"/>
       <c r="E199" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4750,9 +4249,6 @@
           <t>11-D-9819-01</t>
         </is>
       </c>
-      <c r="B200" t="inlineStr"/>
-      <c r="C200" t="inlineStr"/>
-      <c r="D200" t="inlineStr"/>
       <c r="E200" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4770,9 +4266,6 @@
           <t>11-D-9820-01</t>
         </is>
       </c>
-      <c r="B201" t="inlineStr"/>
-      <c r="C201" t="inlineStr"/>
-      <c r="D201" t="inlineStr"/>
       <c r="E201" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4790,9 +4283,6 @@
           <t>11-D-9821-01</t>
         </is>
       </c>
-      <c r="B202" t="inlineStr"/>
-      <c r="C202" t="inlineStr"/>
-      <c r="D202" t="inlineStr"/>
       <c r="E202" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4810,9 +4300,6 @@
           <t>11-D-9824-01</t>
         </is>
       </c>
-      <c r="B203" t="inlineStr"/>
-      <c r="C203" t="inlineStr"/>
-      <c r="D203" t="inlineStr"/>
       <c r="E203" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4830,9 +4317,6 @@
           <t>11-D-9825-01</t>
         </is>
       </c>
-      <c r="B204" t="inlineStr"/>
-      <c r="C204" t="inlineStr"/>
-      <c r="D204" t="inlineStr"/>
       <c r="E204" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4850,9 +4334,6 @@
           <t>11-D-9828-01</t>
         </is>
       </c>
-      <c r="B205" t="inlineStr"/>
-      <c r="C205" t="inlineStr"/>
-      <c r="D205" t="inlineStr"/>
       <c r="E205" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4870,9 +4351,6 @@
           <t>11-D-9829-01</t>
         </is>
       </c>
-      <c r="B206" t="inlineStr"/>
-      <c r="C206" t="inlineStr"/>
-      <c r="D206" t="inlineStr"/>
       <c r="E206" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4890,9 +4368,6 @@
           <t>11-D-9832-01</t>
         </is>
       </c>
-      <c r="B207" t="inlineStr"/>
-      <c r="C207" t="inlineStr"/>
-      <c r="D207" t="inlineStr"/>
       <c r="E207" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4910,9 +4385,6 @@
           <t>11-D-9903-01</t>
         </is>
       </c>
-      <c r="B208" t="inlineStr"/>
-      <c r="C208" t="inlineStr"/>
-      <c r="D208" t="inlineStr"/>
       <c r="E208" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4930,9 +4402,6 @@
           <t>11-D-9978-201</t>
         </is>
       </c>
-      <c r="B209" t="inlineStr"/>
-      <c r="C209" t="inlineStr"/>
-      <c r="D209" t="inlineStr"/>
       <c r="E209" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4950,9 +4419,6 @@
           <t>11-D-9978-202</t>
         </is>
       </c>
-      <c r="B210" t="inlineStr"/>
-      <c r="C210" t="inlineStr"/>
-      <c r="D210" t="inlineStr"/>
       <c r="E210" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4970,9 +4436,6 @@
           <t>11-E-9246-01</t>
         </is>
       </c>
-      <c r="B211" t="inlineStr"/>
-      <c r="C211" t="inlineStr"/>
-      <c r="D211" t="inlineStr"/>
       <c r="E211" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -4990,9 +4453,6 @@
           <t>11-E-9250-01</t>
         </is>
       </c>
-      <c r="B212" t="inlineStr"/>
-      <c r="C212" t="inlineStr"/>
-      <c r="D212" t="inlineStr"/>
       <c r="E212" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5010,9 +4470,6 @@
           <t>11-E-9256-01</t>
         </is>
       </c>
-      <c r="B213" t="inlineStr"/>
-      <c r="C213" t="inlineStr"/>
-      <c r="D213" t="inlineStr"/>
       <c r="E213" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5030,9 +4487,6 @@
           <t>11-E-9258-01</t>
         </is>
       </c>
-      <c r="B214" t="inlineStr"/>
-      <c r="C214" t="inlineStr"/>
-      <c r="D214" t="inlineStr"/>
       <c r="E214" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5050,9 +4504,6 @@
           <t>11-E-9665-01</t>
         </is>
       </c>
-      <c r="B215" t="inlineStr"/>
-      <c r="C215" t="inlineStr"/>
-      <c r="D215" t="inlineStr"/>
       <c r="E215" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5070,9 +4521,6 @@
           <t>11-E-9666-01</t>
         </is>
       </c>
-      <c r="B216" t="inlineStr"/>
-      <c r="C216" t="inlineStr"/>
-      <c r="D216" t="inlineStr"/>
       <c r="E216" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5090,9 +4538,6 @@
           <t>11-E-9667-01</t>
         </is>
       </c>
-      <c r="B217" t="inlineStr"/>
-      <c r="C217" t="inlineStr"/>
-      <c r="D217" t="inlineStr"/>
       <c r="E217" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5110,9 +4555,6 @@
           <t>11-E-9675-01</t>
         </is>
       </c>
-      <c r="B218" t="inlineStr"/>
-      <c r="C218" t="inlineStr"/>
-      <c r="D218" t="inlineStr"/>
       <c r="E218" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5130,9 +4572,6 @@
           <t>11-E-9676-01</t>
         </is>
       </c>
-      <c r="B219" t="inlineStr"/>
-      <c r="C219" t="inlineStr"/>
-      <c r="D219" t="inlineStr"/>
       <c r="E219" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5150,9 +4589,6 @@
           <t>11-E-9740-01</t>
         </is>
       </c>
-      <c r="B220" t="inlineStr"/>
-      <c r="C220" t="inlineStr"/>
-      <c r="D220" t="inlineStr"/>
       <c r="E220" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5170,9 +4606,6 @@
           <t>11-E-9740-04</t>
         </is>
       </c>
-      <c r="B221" t="inlineStr"/>
-      <c r="C221" t="inlineStr"/>
-      <c r="D221" t="inlineStr"/>
       <c r="E221" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5190,9 +4623,6 @@
           <t>11-E-9740-07</t>
         </is>
       </c>
-      <c r="B222" t="inlineStr"/>
-      <c r="C222" t="inlineStr"/>
-      <c r="D222" t="inlineStr"/>
       <c r="E222" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5210,9 +4640,6 @@
           <t>11-E-9741-01</t>
         </is>
       </c>
-      <c r="B223" t="inlineStr"/>
-      <c r="C223" t="inlineStr"/>
-      <c r="D223" t="inlineStr"/>
       <c r="E223" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5230,9 +4657,6 @@
           <t>11-E-9741-04</t>
         </is>
       </c>
-      <c r="B224" t="inlineStr"/>
-      <c r="C224" t="inlineStr"/>
-      <c r="D224" t="inlineStr"/>
       <c r="E224" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5250,9 +4674,6 @@
           <t>11-E-9742-01</t>
         </is>
       </c>
-      <c r="B225" t="inlineStr"/>
-      <c r="C225" t="inlineStr"/>
-      <c r="D225" t="inlineStr"/>
       <c r="E225" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5270,9 +4691,6 @@
           <t>11-E-9742-04</t>
         </is>
       </c>
-      <c r="B226" t="inlineStr"/>
-      <c r="C226" t="inlineStr"/>
-      <c r="D226" t="inlineStr"/>
       <c r="E226" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5290,9 +4708,6 @@
           <t>11-E-9745-01</t>
         </is>
       </c>
-      <c r="B227" t="inlineStr"/>
-      <c r="C227" t="inlineStr"/>
-      <c r="D227" t="inlineStr"/>
       <c r="E227" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5310,9 +4725,6 @@
           <t>11-E-9745-04</t>
         </is>
       </c>
-      <c r="B228" t="inlineStr"/>
-      <c r="C228" t="inlineStr"/>
-      <c r="D228" t="inlineStr"/>
       <c r="E228" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5330,9 +4742,6 @@
           <t>11-E-9745-07</t>
         </is>
       </c>
-      <c r="B229" t="inlineStr"/>
-      <c r="C229" t="inlineStr"/>
-      <c r="D229" t="inlineStr"/>
       <c r="E229" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5350,9 +4759,6 @@
           <t>11-E-9746-01</t>
         </is>
       </c>
-      <c r="B230" t="inlineStr"/>
-      <c r="C230" t="inlineStr"/>
-      <c r="D230" t="inlineStr"/>
       <c r="E230" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5370,9 +4776,6 @@
           <t>11-E-9749-01</t>
         </is>
       </c>
-      <c r="B231" t="inlineStr"/>
-      <c r="C231" t="inlineStr"/>
-      <c r="D231" t="inlineStr"/>
       <c r="E231" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5390,9 +4793,6 @@
           <t>11-E-9752-01</t>
         </is>
       </c>
-      <c r="B232" t="inlineStr"/>
-      <c r="C232" t="inlineStr"/>
-      <c r="D232" t="inlineStr"/>
       <c r="E232" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5410,9 +4810,6 @@
           <t>11-E-9754-01</t>
         </is>
       </c>
-      <c r="B233" t="inlineStr"/>
-      <c r="C233" t="inlineStr"/>
-      <c r="D233" t="inlineStr"/>
       <c r="E233" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5430,9 +4827,6 @@
           <t>11-E-9755-01</t>
         </is>
       </c>
-      <c r="B234" t="inlineStr"/>
-      <c r="C234" t="inlineStr"/>
-      <c r="D234" t="inlineStr"/>
       <c r="E234" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5450,9 +4844,6 @@
           <t>11-E-9756-01</t>
         </is>
       </c>
-      <c r="B235" t="inlineStr"/>
-      <c r="C235" t="inlineStr"/>
-      <c r="D235" t="inlineStr"/>
       <c r="E235" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5470,9 +4861,6 @@
           <t>11-E-9757-01</t>
         </is>
       </c>
-      <c r="B236" t="inlineStr"/>
-      <c r="C236" t="inlineStr"/>
-      <c r="D236" t="inlineStr"/>
       <c r="E236" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5490,9 +4878,6 @@
           <t>11-E-9758-01</t>
         </is>
       </c>
-      <c r="B237" t="inlineStr"/>
-      <c r="C237" t="inlineStr"/>
-      <c r="D237" t="inlineStr"/>
       <c r="E237" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5510,9 +4895,6 @@
           <t>11-E-9759-01</t>
         </is>
       </c>
-      <c r="B238" t="inlineStr"/>
-      <c r="C238" t="inlineStr"/>
-      <c r="D238" t="inlineStr"/>
       <c r="E238" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5530,9 +4912,6 @@
           <t>11-E-9760-01</t>
         </is>
       </c>
-      <c r="B239" t="inlineStr"/>
-      <c r="C239" t="inlineStr"/>
-      <c r="D239" t="inlineStr"/>
       <c r="E239" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5550,9 +4929,6 @@
           <t>11-E-9761-01</t>
         </is>
       </c>
-      <c r="B240" t="inlineStr"/>
-      <c r="C240" t="inlineStr"/>
-      <c r="D240" t="inlineStr"/>
       <c r="E240" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5570,9 +4946,6 @@
           <t>11-E-9762-01</t>
         </is>
       </c>
-      <c r="B241" t="inlineStr"/>
-      <c r="C241" t="inlineStr"/>
-      <c r="D241" t="inlineStr"/>
       <c r="E241" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5590,9 +4963,6 @@
           <t>11-E-9763-01</t>
         </is>
       </c>
-      <c r="B242" t="inlineStr"/>
-      <c r="C242" t="inlineStr"/>
-      <c r="D242" t="inlineStr"/>
       <c r="E242" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5610,9 +4980,6 @@
           <t>11-E-9764-01</t>
         </is>
       </c>
-      <c r="B243" t="inlineStr"/>
-      <c r="C243" t="inlineStr"/>
-      <c r="D243" t="inlineStr"/>
       <c r="E243" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5630,9 +4997,6 @@
           <t>11-E-9767-01</t>
         </is>
       </c>
-      <c r="B244" t="inlineStr"/>
-      <c r="C244" t="inlineStr"/>
-      <c r="D244" t="inlineStr"/>
       <c r="E244" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5650,9 +5014,6 @@
           <t>11-E-9768-01</t>
         </is>
       </c>
-      <c r="B245" t="inlineStr"/>
-      <c r="C245" t="inlineStr"/>
-      <c r="D245" t="inlineStr"/>
       <c r="E245" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5670,9 +5031,6 @@
           <t>11-E-9769-01</t>
         </is>
       </c>
-      <c r="B246" t="inlineStr"/>
-      <c r="C246" t="inlineStr"/>
-      <c r="D246" t="inlineStr"/>
       <c r="E246" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5690,9 +5048,6 @@
           <t>11-E-9772-01</t>
         </is>
       </c>
-      <c r="B247" t="inlineStr"/>
-      <c r="C247" t="inlineStr"/>
-      <c r="D247" t="inlineStr"/>
       <c r="E247" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5710,9 +5065,6 @@
           <t>11-E-9773-01</t>
         </is>
       </c>
-      <c r="B248" t="inlineStr"/>
-      <c r="C248" t="inlineStr"/>
-      <c r="D248" t="inlineStr"/>
       <c r="E248" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5730,9 +5082,6 @@
           <t>11-E-9774-01</t>
         </is>
       </c>
-      <c r="B249" t="inlineStr"/>
-      <c r="C249" t="inlineStr"/>
-      <c r="D249" t="inlineStr"/>
       <c r="E249" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5750,9 +5099,6 @@
           <t>11-E-9839-01</t>
         </is>
       </c>
-      <c r="B250" t="inlineStr"/>
-      <c r="C250" t="inlineStr"/>
-      <c r="D250" t="inlineStr"/>
       <c r="E250" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5770,9 +5116,6 @@
           <t>11-E-9839-04</t>
         </is>
       </c>
-      <c r="B251" t="inlineStr"/>
-      <c r="C251" t="inlineStr"/>
-      <c r="D251" t="inlineStr"/>
       <c r="E251" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5790,9 +5133,6 @@
           <t>11-E-9846-01</t>
         </is>
       </c>
-      <c r="B252" t="inlineStr"/>
-      <c r="C252" t="inlineStr"/>
-      <c r="D252" t="inlineStr"/>
       <c r="E252" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5810,9 +5150,6 @@
           <t>11-E-9851-01</t>
         </is>
       </c>
-      <c r="B253" t="inlineStr"/>
-      <c r="C253" t="inlineStr"/>
-      <c r="D253" t="inlineStr"/>
       <c r="E253" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5830,9 +5167,6 @@
           <t>11-E-9851-02</t>
         </is>
       </c>
-      <c r="B254" t="inlineStr"/>
-      <c r="C254" t="inlineStr"/>
-      <c r="D254" t="inlineStr"/>
       <c r="E254" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -5850,9 +5184,6 @@
           <t>11-E-9870-02</t>
         </is>
       </c>
-      <c r="B255" t="inlineStr"/>
-      <c r="C255" t="inlineStr"/>
-      <c r="D255" t="inlineStr"/>
       <c r="E255" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5870,9 +5201,6 @@
           <t>11-E-9871-02</t>
         </is>
       </c>
-      <c r="B256" t="inlineStr"/>
-      <c r="C256" t="inlineStr"/>
-      <c r="D256" t="inlineStr"/>
       <c r="E256" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5890,9 +5218,6 @@
           <t>11-E-9872-02</t>
         </is>
       </c>
-      <c r="B257" t="inlineStr"/>
-      <c r="C257" t="inlineStr"/>
-      <c r="D257" t="inlineStr"/>
       <c r="E257" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5910,9 +5235,6 @@
           <t>11-E-9892-01</t>
         </is>
       </c>
-      <c r="B258" t="inlineStr"/>
-      <c r="C258" t="inlineStr"/>
-      <c r="D258" t="inlineStr"/>
       <c r="E258" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5930,9 +5252,6 @@
           <t>11-E-9892-03</t>
         </is>
       </c>
-      <c r="B259" t="inlineStr"/>
-      <c r="C259" t="inlineStr"/>
-      <c r="D259" t="inlineStr"/>
       <c r="E259" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5950,9 +5269,6 @@
           <t>11-E-9893-01</t>
         </is>
       </c>
-      <c r="B260" t="inlineStr"/>
-      <c r="C260" t="inlineStr"/>
-      <c r="D260" t="inlineStr"/>
       <c r="E260" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5970,9 +5286,6 @@
           <t>11-E-9893-03</t>
         </is>
       </c>
-      <c r="B261" t="inlineStr"/>
-      <c r="C261" t="inlineStr"/>
-      <c r="D261" t="inlineStr"/>
       <c r="E261" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -5990,9 +5303,6 @@
           <t>11-E-9894-01</t>
         </is>
       </c>
-      <c r="B262" t="inlineStr"/>
-      <c r="C262" t="inlineStr"/>
-      <c r="D262" t="inlineStr"/>
       <c r="E262" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6010,9 +5320,6 @@
           <t>11-E-9894-03</t>
         </is>
       </c>
-      <c r="B263" t="inlineStr"/>
-      <c r="C263" t="inlineStr"/>
-      <c r="D263" t="inlineStr"/>
       <c r="E263" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6030,9 +5337,6 @@
           <t>11-E-9894-09</t>
         </is>
       </c>
-      <c r="B264" t="inlineStr"/>
-      <c r="C264" t="inlineStr"/>
-      <c r="D264" t="inlineStr"/>
       <c r="E264" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6050,9 +5354,6 @@
           <t>11-E-9895-01</t>
         </is>
       </c>
-      <c r="B265" t="inlineStr"/>
-      <c r="C265" t="inlineStr"/>
-      <c r="D265" t="inlineStr"/>
       <c r="E265" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6070,9 +5371,6 @@
           <t>11-E-9896-01</t>
         </is>
       </c>
-      <c r="B266" t="inlineStr"/>
-      <c r="C266" t="inlineStr"/>
-      <c r="D266" t="inlineStr"/>
       <c r="E266" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6090,9 +5388,6 @@
           <t>11-E-9897-01</t>
         </is>
       </c>
-      <c r="B267" t="inlineStr"/>
-      <c r="C267" t="inlineStr"/>
-      <c r="D267" t="inlineStr"/>
       <c r="E267" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6110,9 +5405,6 @@
           <t>11-E-9897-03</t>
         </is>
       </c>
-      <c r="B268" t="inlineStr"/>
-      <c r="C268" t="inlineStr"/>
-      <c r="D268" t="inlineStr"/>
       <c r="E268" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6130,9 +5422,6 @@
           <t>11-E-9898-01</t>
         </is>
       </c>
-      <c r="B269" t="inlineStr"/>
-      <c r="C269" t="inlineStr"/>
-      <c r="D269" t="inlineStr"/>
       <c r="E269" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6150,9 +5439,6 @@
           <t>11-E-9898-03</t>
         </is>
       </c>
-      <c r="B270" t="inlineStr"/>
-      <c r="C270" t="inlineStr"/>
-      <c r="D270" t="inlineStr"/>
       <c r="E270" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6170,9 +5456,6 @@
           <t>11-E-9899-01</t>
         </is>
       </c>
-      <c r="B271" t="inlineStr"/>
-      <c r="C271" t="inlineStr"/>
-      <c r="D271" t="inlineStr"/>
       <c r="E271" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6190,9 +5473,6 @@
           <t>11-E-9900-01</t>
         </is>
       </c>
-      <c r="B272" t="inlineStr"/>
-      <c r="C272" t="inlineStr"/>
-      <c r="D272" t="inlineStr"/>
       <c r="E272" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6210,9 +5490,6 @@
           <t>11-E-9900-03</t>
         </is>
       </c>
-      <c r="B273" t="inlineStr"/>
-      <c r="C273" t="inlineStr"/>
-      <c r="D273" t="inlineStr"/>
       <c r="E273" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6230,9 +5507,6 @@
           <t>11-E-9900-09</t>
         </is>
       </c>
-      <c r="B274" t="inlineStr"/>
-      <c r="C274" t="inlineStr"/>
-      <c r="D274" t="inlineStr"/>
       <c r="E274" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6250,9 +5524,6 @@
           <t>11-E-9901-01</t>
         </is>
       </c>
-      <c r="B275" t="inlineStr"/>
-      <c r="C275" t="inlineStr"/>
-      <c r="D275" t="inlineStr"/>
       <c r="E275" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6270,9 +5541,6 @@
           <t>11-E-9902-01</t>
         </is>
       </c>
-      <c r="B276" t="inlineStr"/>
-      <c r="C276" t="inlineStr"/>
-      <c r="D276" t="inlineStr"/>
       <c r="E276" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6290,9 +5558,6 @@
           <t>11-E-9903-01</t>
         </is>
       </c>
-      <c r="B277" t="inlineStr"/>
-      <c r="C277" t="inlineStr"/>
-      <c r="D277" t="inlineStr"/>
       <c r="E277" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6310,9 +5575,6 @@
           <t>11-E-9909-02</t>
         </is>
       </c>
-      <c r="B278" t="inlineStr"/>
-      <c r="C278" t="inlineStr"/>
-      <c r="D278" t="inlineStr"/>
       <c r="E278" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6330,9 +5592,6 @@
           <t>11-E-9910-02</t>
         </is>
       </c>
-      <c r="B279" t="inlineStr"/>
-      <c r="C279" t="inlineStr"/>
-      <c r="D279" t="inlineStr"/>
       <c r="E279" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6350,9 +5609,6 @@
           <t>11-E-9911-02</t>
         </is>
       </c>
-      <c r="B280" t="inlineStr"/>
-      <c r="C280" t="inlineStr"/>
-      <c r="D280" t="inlineStr"/>
       <c r="E280" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6370,9 +5626,6 @@
           <t>11-F-9005-01</t>
         </is>
       </c>
-      <c r="B281" t="inlineStr"/>
-      <c r="C281" t="inlineStr"/>
-      <c r="D281" t="inlineStr"/>
       <c r="E281" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6390,9 +5643,6 @@
           <t>11-F-9006-01</t>
         </is>
       </c>
-      <c r="B282" t="inlineStr"/>
-      <c r="C282" t="inlineStr"/>
-      <c r="D282" t="inlineStr"/>
       <c r="E282" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6410,9 +5660,6 @@
           <t>11-F-9276-01</t>
         </is>
       </c>
-      <c r="B283" t="inlineStr"/>
-      <c r="C283" t="inlineStr"/>
-      <c r="D283" t="inlineStr"/>
       <c r="E283" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6590,9 +5837,6 @@
           <t>12-6010-08</t>
         </is>
       </c>
-      <c r="B289" t="inlineStr"/>
-      <c r="C289" t="inlineStr"/>
-      <c r="D289" t="inlineStr"/>
       <c r="E289" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6674,9 +5918,6 @@
           <t>12-6010-12</t>
         </is>
       </c>
-      <c r="B292" t="inlineStr"/>
-      <c r="C292" t="inlineStr"/>
-      <c r="D292" t="inlineStr"/>
       <c r="E292" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6736,7 +5977,6 @@
           <t>14GA</t>
         </is>
       </c>
-      <c r="D294" t="inlineStr"/>
       <c r="E294" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -6764,7 +6004,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D295" t="inlineStr"/>
       <c r="E295" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -6846,9 +6085,6 @@
           <t>12-6355-38</t>
         </is>
       </c>
-      <c r="B298" t="inlineStr"/>
-      <c r="C298" t="inlineStr"/>
-      <c r="D298" t="inlineStr"/>
       <c r="E298" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -6876,7 +6112,6 @@
           <t>14GA</t>
         </is>
       </c>
-      <c r="D299" t="inlineStr"/>
       <c r="E299" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -6899,8 +6134,6 @@
           <t>12-A-6199-01-(12gacr ANSI-61) - K48 - V3-R0</t>
         </is>
       </c>
-      <c r="C300" t="inlineStr"/>
-      <c r="D300" t="inlineStr"/>
       <c r="E300" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -7014,9 +6247,6 @@
           <t>12-A-6348-03</t>
         </is>
       </c>
-      <c r="B304" t="inlineStr"/>
-      <c r="C304" t="inlineStr"/>
-      <c r="D304" t="inlineStr"/>
       <c r="E304" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -7258,9 +6488,6 @@
           <t>12-D-6013-01</t>
         </is>
       </c>
-      <c r="B312" t="inlineStr"/>
-      <c r="C312" t="inlineStr"/>
-      <c r="D312" t="inlineStr"/>
       <c r="E312" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -7288,7 +6515,6 @@
           <t>10GA</t>
         </is>
       </c>
-      <c r="D313" t="inlineStr"/>
       <c r="E313" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -7316,7 +6542,6 @@
           <t>10GA</t>
         </is>
       </c>
-      <c r="D314" t="inlineStr"/>
       <c r="E314" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -7339,8 +6564,6 @@
           <t>12-D-6030-10 - PLATE TOP GALVANIZADO</t>
         </is>
       </c>
-      <c r="C315" t="inlineStr"/>
-      <c r="D315" t="inlineStr"/>
       <c r="E315" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -7422,9 +6645,6 @@
           <t>12-D-6047-09</t>
         </is>
       </c>
-      <c r="B318" t="inlineStr"/>
-      <c r="C318" t="inlineStr"/>
-      <c r="D318" t="inlineStr"/>
       <c r="E318" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -7474,9 +6694,6 @@
           <t>12-D-6066-01</t>
         </is>
       </c>
-      <c r="B320" t="inlineStr"/>
-      <c r="C320" t="inlineStr"/>
-      <c r="D320" t="inlineStr"/>
       <c r="E320" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -7494,9 +6711,6 @@
           <t>12-D-6075-01</t>
         </is>
       </c>
-      <c r="B321" t="inlineStr"/>
-      <c r="C321" t="inlineStr"/>
-      <c r="D321" t="inlineStr"/>
       <c r="E321" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -7546,9 +6760,6 @@
           <t>12-D-6079-05</t>
         </is>
       </c>
-      <c r="B323" t="inlineStr"/>
-      <c r="C323" t="inlineStr"/>
-      <c r="D323" t="inlineStr"/>
       <c r="E323" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -7635,8 +6846,6 @@
           <t>12-D-6081-05-(16gacr ANSI-61) - K48 - V2-R0</t>
         </is>
       </c>
-      <c r="C326" t="inlineStr"/>
-      <c r="D326" t="inlineStr"/>
       <c r="E326" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -7760,7 +6969,6 @@
           <t>16GACR</t>
         </is>
       </c>
-      <c r="D330" t="inlineStr"/>
       <c r="E330" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -7906,9 +7114,6 @@
           <t>12-D-6087-07</t>
         </is>
       </c>
-      <c r="B335" t="inlineStr"/>
-      <c r="C335" t="inlineStr"/>
-      <c r="D335" t="inlineStr"/>
       <c r="E335" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -7931,8 +7136,6 @@
           <t>12-D-6088-06-(16gacr ANSI-61) - K48 - V2-R0</t>
         </is>
       </c>
-      <c r="C336" t="inlineStr"/>
-      <c r="D336" t="inlineStr"/>
       <c r="E336" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -7987,8 +7190,6 @@
           <t>12-D-6089-01-(16gacr ANSI-61) - K48 - V0-R0</t>
         </is>
       </c>
-      <c r="C338" t="inlineStr"/>
-      <c r="D338" t="inlineStr"/>
       <c r="E338" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -8038,9 +7239,6 @@
           <t>12-D-6090-06</t>
         </is>
       </c>
-      <c r="B340" t="inlineStr"/>
-      <c r="C340" t="inlineStr"/>
-      <c r="D340" t="inlineStr"/>
       <c r="E340" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -8058,9 +7256,6 @@
           <t>12-D-6090-07</t>
         </is>
       </c>
-      <c r="B341" t="inlineStr"/>
-      <c r="C341" t="inlineStr"/>
-      <c r="D341" t="inlineStr"/>
       <c r="E341" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -8083,8 +7278,6 @@
           <t>12-D-6091-01-(16gacr ANSI-61) - K48 - V1-R0</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr"/>
-      <c r="D342" t="inlineStr"/>
       <c r="E342" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -8230,9 +7423,6 @@
           <t>12-D-6099-01</t>
         </is>
       </c>
-      <c r="B347" t="inlineStr"/>
-      <c r="C347" t="inlineStr"/>
-      <c r="D347" t="inlineStr"/>
       <c r="E347" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -8538,9 +7728,6 @@
           <t>12-D-6107-02</t>
         </is>
       </c>
-      <c r="B357" t="inlineStr"/>
-      <c r="C357" t="inlineStr"/>
-      <c r="D357" t="inlineStr"/>
       <c r="E357" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -8600,7 +7787,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D359" t="inlineStr"/>
       <c r="E359" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -8628,7 +7814,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D360" t="inlineStr"/>
       <c r="E360" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -8710,13 +7895,11 @@
           <t>12-D-6412-01</t>
         </is>
       </c>
-      <c r="B363" t="inlineStr"/>
       <c r="C363" t="inlineStr">
         <is>
           <t>14GACR</t>
         </is>
       </c>
-      <c r="D363" t="inlineStr"/>
       <c r="E363" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -8734,13 +7917,11 @@
           <t>12-D-6412-03</t>
         </is>
       </c>
-      <c r="B364" t="inlineStr"/>
       <c r="C364" t="inlineStr">
         <is>
           <t>14GACR</t>
         </is>
       </c>
-      <c r="D364" t="inlineStr"/>
       <c r="E364" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -8758,13 +7939,11 @@
           <t>12-D-6412-05</t>
         </is>
       </c>
-      <c r="B365" t="inlineStr"/>
       <c r="C365" t="inlineStr">
         <is>
           <t>14GACR</t>
         </is>
       </c>
-      <c r="D365" t="inlineStr"/>
       <c r="E365" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -8883,8 +8062,6 @@
           <t>16-6082-01-(16gacr ANSI-61) - K48 - V0-R0</t>
         </is>
       </c>
-      <c r="C369" t="inlineStr"/>
-      <c r="D369" t="inlineStr"/>
       <c r="E369" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -8902,13 +8079,11 @@
           <t>16-A-6001-01</t>
         </is>
       </c>
-      <c r="B370" t="inlineStr"/>
       <c r="C370" t="inlineStr">
         <is>
           <t>12GACR</t>
         </is>
       </c>
-      <c r="D370" t="inlineStr"/>
       <c r="E370" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -9374,9 +8549,6 @@
           <t>P15324-19</t>
         </is>
       </c>
-      <c r="B385" t="inlineStr"/>
-      <c r="C385" t="inlineStr"/>
-      <c r="D385" t="inlineStr"/>
       <c r="E385" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -9394,9 +8566,6 @@
           <t>P15899-10</t>
         </is>
       </c>
-      <c r="B386" t="inlineStr"/>
-      <c r="C386" t="inlineStr"/>
-      <c r="D386" t="inlineStr"/>
       <c r="E386" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -9424,7 +8593,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D387" t="inlineStr"/>
       <c r="E387" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -9932,7 +9100,6 @@
           <t>14GA</t>
         </is>
       </c>
-      <c r="D403" t="inlineStr"/>
       <c r="E403" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -10024,7 +9191,6 @@
           <t>10GA</t>
         </is>
       </c>
-      <c r="D406" t="inlineStr"/>
       <c r="E406" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -10052,7 +9218,6 @@
           <t>10GA</t>
         </is>
       </c>
-      <c r="D407" t="inlineStr"/>
       <c r="E407" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -10080,7 +9245,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D408" t="inlineStr"/>
       <c r="E408" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -10268,7 +9432,6 @@
           <t>10GA</t>
         </is>
       </c>
-      <c r="D414" t="inlineStr"/>
       <c r="E414" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -10328,7 +9491,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D416" t="inlineStr"/>
       <c r="E416" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -10356,7 +9518,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D417" t="inlineStr"/>
       <c r="E417" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -10384,7 +9545,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D418" t="inlineStr"/>
       <c r="E418" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -10412,7 +9572,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D419" t="inlineStr"/>
       <c r="E419" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -10440,7 +9599,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D420" t="inlineStr"/>
       <c r="E420" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -10458,9 +9616,6 @@
           <t>P20553-09</t>
         </is>
       </c>
-      <c r="B421" t="inlineStr"/>
-      <c r="C421" t="inlineStr"/>
-      <c r="D421" t="inlineStr"/>
       <c r="E421" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -10478,9 +9633,6 @@
           <t>P20557-20</t>
         </is>
       </c>
-      <c r="B422" t="inlineStr"/>
-      <c r="C422" t="inlineStr"/>
-      <c r="D422" t="inlineStr"/>
       <c r="E422" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -10498,9 +9650,6 @@
           <t>P20557-21</t>
         </is>
       </c>
-      <c r="B423" t="inlineStr"/>
-      <c r="C423" t="inlineStr"/>
-      <c r="D423" t="inlineStr"/>
       <c r="E423" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -10518,9 +9667,6 @@
           <t>P20593-15</t>
         </is>
       </c>
-      <c r="B424" t="inlineStr"/>
-      <c r="C424" t="inlineStr"/>
-      <c r="D424" t="inlineStr"/>
       <c r="E424" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -10538,9 +9684,6 @@
           <t>P20596-21</t>
         </is>
       </c>
-      <c r="B425" t="inlineStr"/>
-      <c r="C425" t="inlineStr"/>
-      <c r="D425" t="inlineStr"/>
       <c r="E425" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -10558,9 +9701,6 @@
           <t>P20596-22</t>
         </is>
       </c>
-      <c r="B426" t="inlineStr"/>
-      <c r="C426" t="inlineStr"/>
-      <c r="D426" t="inlineStr"/>
       <c r="E426" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -10610,9 +9750,6 @@
           <t>P8815-03</t>
         </is>
       </c>
-      <c r="B428" t="inlineStr"/>
-      <c r="C428" t="inlineStr"/>
-      <c r="D428" t="inlineStr"/>
       <c r="E428" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -10630,9 +9767,6 @@
           <t>P8815-04</t>
         </is>
       </c>
-      <c r="B429" t="inlineStr"/>
-      <c r="C429" t="inlineStr"/>
-      <c r="D429" t="inlineStr"/>
       <c r="E429" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -10650,9 +9784,6 @@
           <t>P9711-08</t>
         </is>
       </c>
-      <c r="B430" t="inlineStr"/>
-      <c r="C430" t="inlineStr"/>
-      <c r="D430" t="inlineStr"/>
       <c r="E430" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -10670,9 +9801,6 @@
           <t>P9711-081</t>
         </is>
       </c>
-      <c r="B431" t="inlineStr"/>
-      <c r="C431" t="inlineStr"/>
-      <c r="D431" t="inlineStr"/>
       <c r="E431" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -10690,9 +9818,6 @@
           <t>PP10218-13</t>
         </is>
       </c>
-      <c r="B432" t="inlineStr"/>
-      <c r="C432" t="inlineStr"/>
-      <c r="D432" t="inlineStr"/>
       <c r="E432" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -10816,7 +9941,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D436" t="inlineStr"/>
       <c r="E436" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -10844,7 +9968,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D437" t="inlineStr"/>
       <c r="E437" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -10872,7 +9995,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D438" t="inlineStr"/>
       <c r="E438" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -10900,7 +10022,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D439" t="inlineStr"/>
       <c r="E439" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -10923,8 +10044,6 @@
           <t>PP14023-01-(16gacr ANSI-61) - K48 - V0-R0</t>
         </is>
       </c>
-      <c r="C440" t="inlineStr"/>
-      <c r="D440" t="inlineStr"/>
       <c r="E440" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -10984,7 +10103,6 @@
           <t>10GA</t>
         </is>
       </c>
-      <c r="D442" t="inlineStr"/>
       <c r="E442" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -11034,9 +10152,6 @@
           <t>PP14873-01</t>
         </is>
       </c>
-      <c r="B444" t="inlineStr"/>
-      <c r="C444" t="inlineStr"/>
-      <c r="D444" t="inlineStr"/>
       <c r="E444" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -11054,9 +10169,6 @@
           <t>PP14873-02</t>
         </is>
       </c>
-      <c r="B445" t="inlineStr"/>
-      <c r="C445" t="inlineStr"/>
-      <c r="D445" t="inlineStr"/>
       <c r="E445" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -11298,9 +10410,6 @@
           <t>PP19187-05</t>
         </is>
       </c>
-      <c r="B453" t="inlineStr"/>
-      <c r="C453" t="inlineStr"/>
-      <c r="D453" t="inlineStr"/>
       <c r="E453" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -11392,7 +10501,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D456" t="inlineStr"/>
       <c r="E456" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -11420,7 +10528,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D457" t="inlineStr"/>
       <c r="E457" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -11448,7 +10555,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D458" t="inlineStr"/>
       <c r="E458" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -11476,7 +10582,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D459" t="inlineStr"/>
       <c r="E459" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -11504,7 +10609,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D460" t="inlineStr"/>
       <c r="E460" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -11532,7 +10636,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D461" t="inlineStr"/>
       <c r="E461" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -11560,7 +10663,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D462" t="inlineStr"/>
       <c r="E462" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -11588,7 +10690,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D463" t="inlineStr"/>
       <c r="E463" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -11616,7 +10717,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D464" t="inlineStr"/>
       <c r="E464" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -11644,7 +10744,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D465" t="inlineStr"/>
       <c r="E465" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -11662,9 +10761,6 @@
           <t>PP20825-02</t>
         </is>
       </c>
-      <c r="B466" t="inlineStr"/>
-      <c r="C466" t="inlineStr"/>
-      <c r="D466" t="inlineStr"/>
       <c r="E466" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -11682,9 +10778,6 @@
           <t>PP21139-081</t>
         </is>
       </c>
-      <c r="B467" t="inlineStr"/>
-      <c r="C467" t="inlineStr"/>
-      <c r="D467" t="inlineStr"/>
       <c r="E467" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -11702,9 +10795,6 @@
           <t>PP21139-082</t>
         </is>
       </c>
-      <c r="B468" t="inlineStr"/>
-      <c r="C468" t="inlineStr"/>
-      <c r="D468" t="inlineStr"/>
       <c r="E468" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -11722,9 +10812,6 @@
           <t>PP21139-091</t>
         </is>
       </c>
-      <c r="B469" t="inlineStr"/>
-      <c r="C469" t="inlineStr"/>
-      <c r="D469" t="inlineStr"/>
       <c r="E469" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -11742,9 +10829,6 @@
           <t>PP21139-092</t>
         </is>
       </c>
-      <c r="B470" t="inlineStr"/>
-      <c r="C470" t="inlineStr"/>
-      <c r="D470" t="inlineStr"/>
       <c r="E470" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -12082,9 +11166,6 @@
           <t>PP6868-113</t>
         </is>
       </c>
-      <c r="B481" t="inlineStr"/>
-      <c r="C481" t="inlineStr"/>
-      <c r="D481" t="inlineStr"/>
       <c r="E481" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -12102,9 +11183,6 @@
           <t>PP7114-72</t>
         </is>
       </c>
-      <c r="B482" t="inlineStr"/>
-      <c r="C482" t="inlineStr"/>
-      <c r="D482" t="inlineStr"/>
       <c r="E482" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -12218,9 +11296,6 @@
           <t>PP8192-05</t>
         </is>
       </c>
-      <c r="B486" t="inlineStr"/>
-      <c r="C486" t="inlineStr"/>
-      <c r="D486" t="inlineStr"/>
       <c r="E486" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -12238,10 +11313,6 @@
           <t>11-D-6195-05</t>
         </is>
       </c>
-      <c r="B487" t="inlineStr"/>
-      <c r="C487" t="inlineStr"/>
-      <c r="D487" t="inlineStr"/>
-      <c r="E487" t="inlineStr"/>
       <c r="F487" t="inlineStr">
         <is>
           <t>SWB00084</t>
@@ -12254,10 +11325,6 @@
           <t>11-D-6195-06</t>
         </is>
       </c>
-      <c r="B488" t="inlineStr"/>
-      <c r="C488" t="inlineStr"/>
-      <c r="D488" t="inlineStr"/>
-      <c r="E488" t="inlineStr"/>
       <c r="F488" t="inlineStr">
         <is>
           <t>SWB01454</t>
@@ -12270,10 +11337,6 @@
           <t>P9014-102</t>
         </is>
       </c>
-      <c r="B489" t="inlineStr"/>
-      <c r="C489" t="inlineStr"/>
-      <c r="D489" t="inlineStr"/>
-      <c r="E489" t="inlineStr"/>
       <c r="F489" t="inlineStr">
         <is>
           <t>SWB01512</t>
@@ -12520,7 +11583,6 @@
           <t>12GA</t>
         </is>
       </c>
-      <c r="D497" t="inlineStr"/>
       <c r="E497" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -12735,8 +11797,6 @@
           <t>12-D-6083-03</t>
         </is>
       </c>
-      <c r="C504" t="inlineStr"/>
-      <c r="D504" t="inlineStr"/>
       <c r="E504" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -12759,8 +11819,6 @@
           <t>12-D-6106-01</t>
         </is>
       </c>
-      <c r="C505" t="inlineStr"/>
-      <c r="D505" t="inlineStr"/>
       <c r="E505" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -12783,8 +11841,6 @@
           <t>PP21139-092 TRTO - Proyecto TORONTO</t>
         </is>
       </c>
-      <c r="C506" t="inlineStr"/>
-      <c r="D506" t="inlineStr"/>
       <c r="E506" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -12807,8 +11863,6 @@
           <t>PP21139-092 TRT0 - Proyecto TORONTO</t>
         </is>
       </c>
-      <c r="C507" t="inlineStr"/>
-      <c r="D507" t="inlineStr"/>
       <c r="E507" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -12831,8 +11885,6 @@
           <t>P9711-081 TRTO 2 - Proyecto TORONTO</t>
         </is>
       </c>
-      <c r="C508" t="inlineStr"/>
-      <c r="D508" t="inlineStr"/>
       <c r="E508" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -12855,8 +11907,6 @@
           <t>P9711-081 TRT0 2 - Proyecto TORONTO</t>
         </is>
       </c>
-      <c r="C509" t="inlineStr"/>
-      <c r="D509" t="inlineStr"/>
       <c r="E509" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -12879,8 +11929,6 @@
           <t>P7911-081 TRTO 1 - Proyecto TORONTO</t>
         </is>
       </c>
-      <c r="C510" t="inlineStr"/>
-      <c r="D510" t="inlineStr"/>
       <c r="E510" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -12903,8 +11951,6 @@
           <t>P7911-081 TRT0 1 - Proyecto TORONTO</t>
         </is>
       </c>
-      <c r="C511" t="inlineStr"/>
-      <c r="D511" t="inlineStr"/>
       <c r="E511" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -12927,8 +11973,6 @@
           <t>P9711-081 TRTO 1 - Proyecto TORONTO</t>
         </is>
       </c>
-      <c r="C512" t="inlineStr"/>
-      <c r="D512" t="inlineStr"/>
       <c r="E512" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -12951,8 +11995,6 @@
           <t>P9711-081 TRT0 1 - Proyecto TORONTO</t>
         </is>
       </c>
-      <c r="C513" t="inlineStr"/>
-      <c r="D513" t="inlineStr"/>
       <c r="E513" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -13135,8 +12177,6 @@
           <t>P9711-081 TRTO - Proyecto TORONTO</t>
         </is>
       </c>
-      <c r="C519" t="inlineStr"/>
-      <c r="D519" t="inlineStr"/>
       <c r="E519" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -13159,8 +12199,6 @@
           <t>P9711-081 TRT0 - Proyecto TORONTO</t>
         </is>
       </c>
-      <c r="C520" t="inlineStr"/>
-      <c r="D520" t="inlineStr"/>
       <c r="E520" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -13183,8 +12221,6 @@
           <t>PP21139-081 TRTO - Proyecto TORONTO</t>
         </is>
       </c>
-      <c r="C521" t="inlineStr"/>
-      <c r="D521" t="inlineStr"/>
       <c r="E521" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -13207,8 +12243,6 @@
           <t>PP21139-081 TRT0 - Proyecto TORONTO</t>
         </is>
       </c>
-      <c r="C522" t="inlineStr"/>
-      <c r="D522" t="inlineStr"/>
       <c r="E522" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -13231,8 +12265,6 @@
           <t>11-C-9778-01 TRTO - Proyecto TORONTO</t>
         </is>
       </c>
-      <c r="C523" t="inlineStr"/>
-      <c r="D523" t="inlineStr"/>
       <c r="E523" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -13255,8 +12287,6 @@
           <t>11-C-9778-01 TRT0 - Proyecto TORONTO</t>
         </is>
       </c>
-      <c r="C524" t="inlineStr"/>
-      <c r="D524" t="inlineStr"/>
       <c r="E524" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -13279,8 +12309,16 @@
           <t>12-D-6030-07 - PLATE TOP GALVANIZADO</t>
         </is>
       </c>
-      <c r="C525" t="inlineStr"/>
-      <c r="D525" t="inlineStr"/>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E525" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -13303,8 +12341,16 @@
           <t>12-D-6030-08 - PLATE TOP GALVANIZADO</t>
         </is>
       </c>
-      <c r="C526" t="inlineStr"/>
-      <c r="D526" t="inlineStr"/>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E526" t="inlineStr">
         <is>
           <t>Galvanizado</t>
@@ -13319,16 +12365,19 @@
     <row r="527">
       <c r="A527" t="inlineStr">
         <is>
-          <t>11-A-9581-01 TRTO</t>
+          <t>11-A-9581-01 TRTC</t>
         </is>
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>11-A-9581-01 TRTO</t>
-        </is>
-      </c>
-      <c r="C527" t="inlineStr"/>
-      <c r="D527" t="inlineStr"/>
+          <t>11-A-9581-01 TRTC - RUN-BACK LUG BRACKET (TORONTO)</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Decapado CAL 16 (16 GA)</t>
+        </is>
+      </c>
       <c r="E527" t="inlineStr">
         <is>
           <t>Ansi 61</t>
@@ -13336,35 +12385,175 @@
       </c>
       <c r="F527" t="inlineStr">
         <is>
-          <t>11-A-9581-01 TRTO</t>
+          <t>ISSIV00746</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" t="inlineStr">
         <is>
+          <t>11-A-9581-01 TRTO</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>11-A-9581-01 TRTO - RUN-BACK LUG BRACKET (TORONTO)</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Decapado CAL 16 (16 GA)</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>Ansi 61</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>ISSIV00746</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>11-A-9581-01 TRT0</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>11-A-9581-01 TRT0 - RUN-BACK LUG BRACKET (TORONTO)</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>Decapado CAL 16 (16 GA)</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>Ansi 61</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>ISSIV00746</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>11-E-9770-02 TRTC</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>11-E-9770-02 TRTC - Proyecto TORONTO</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>Galvanizado</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>11-E-9770-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>11-E-9770-02 TRTO</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>11-E-9770-02 TRTO - Proyecto TORONTO</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>Galvanizado</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>11-E-9770-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>11-E-9770-02 TRT0</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>11-E-9770-02 TRT0 - Proyecto TORONTO</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>Galvanizado</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>11-E-9770-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>11-E-9770-02</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>11-E-9770-02 - Proyecto TORONTO</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>Galvanizado</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>11-E-9770-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
           <t>12-D-6091-07</t>
         </is>
       </c>
-      <c r="B528" t="inlineStr">
+      <c r="B534" t="inlineStr">
         <is>
           <t>12-D-6091-07</t>
         </is>
       </c>
-      <c r="C528" t="inlineStr"/>
-      <c r="D528" t="inlineStr"/>
-      <c r="E528" t="inlineStr">
-        <is>
-          <t>Ansi 61</t>
-        </is>
-      </c>
-      <c r="F528" t="inlineStr">
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>Ansi 61</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
         <is>
           <t>12-D-6091-07</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>